<commit_message>
Update version and enhance authentication requirements
</commit_message>
<xml_diff>
--- a/docs/Data Model/data-model-spec.xlsx
+++ b/docs/Data Model/data-model-spec.xlsx
@@ -10,7 +10,8 @@
     <sheet name="Indexes" sheetId="1" state="visible" r:id="rId1"/>
     <sheet name="Constraints" sheetId="2" state="visible" r:id="rId2"/>
     <sheet name="Foreign Keys" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Enumerations" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Migration" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Enumerations" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -437,7 +438,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E24"/>
+  <dimension ref="A1:E27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="44" customWidth="1" min="1" max="1"/>
@@ -670,10 +671,14 @@
           <t>Id</t>
         </is>
       </c>
-      <c r="C13" s="3" t="inlineStr"/>
+      <c r="C13" s="3" t="inlineStr">
+        <is>
+          <t>nonclustered</t>
+        </is>
+      </c>
       <c r="D13" s="3" t="inlineStr">
         <is>
-          <t>Guid key</t>
+          <t>Guid key. A random GUID would scatter inserts across the table, so the table is clustered on IX_Users_CreatedUtc instead</t>
         </is>
       </c>
       <c r="E13" s="3" t="inlineStr"/>
@@ -681,35 +686,35 @@
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>UX_Users_NormalizedUserName</t>
+          <t>IX_Users_CreatedUtc</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>NormalizedUserName</t>
+          <t>CreatedUtc, Id</t>
         </is>
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
-          <t>unique</t>
+          <t>clustered</t>
         </is>
       </c>
       <c r="D14" s="3" t="inlineStr">
         <is>
-          <t>Identity's lookup path</t>
-        </is>
-      </c>
-      <c r="E14" s="3" t="inlineStr"/>
+          <t>Keeps inserts appending instead of scattering</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>UX_Users_NormalizedEmail</t>
+          <t>UX_Users_NormalizedUserName</t>
         </is>
       </c>
       <c r="B15" s="3" t="inlineStr">
         <is>
-          <t>NormalizedEmail</t>
+          <t>NormalizedUserName</t>
         </is>
       </c>
       <c r="C15" s="3" t="inlineStr">
@@ -719,7 +724,7 @@
       </c>
       <c r="D15" s="3" t="inlineStr">
         <is>
-          <t>Email is the login</t>
+          <t>Identity's lookup path</t>
         </is>
       </c>
       <c r="E15" s="3" t="inlineStr"/>
@@ -727,18 +732,22 @@
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t>PK_Roles</t>
+          <t>UX_Users_NormalizedEmail</t>
         </is>
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>Id</t>
-        </is>
-      </c>
-      <c r="C16" s="3" t="inlineStr"/>
+          <t>NormalizedEmail</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>unique</t>
+        </is>
+      </c>
       <c r="D16" s="3" t="inlineStr">
         <is>
-          <t>Guid key</t>
+          <t>Email is the login</t>
         </is>
       </c>
       <c r="E16" s="3" t="inlineStr"/>
@@ -746,22 +755,18 @@
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
-          <t>UX_Roles_NormalizedName</t>
+          <t>PK_Roles</t>
         </is>
       </c>
       <c r="B17" s="3" t="inlineStr">
         <is>
-          <t>NormalizedName</t>
-        </is>
-      </c>
-      <c r="C17" s="3" t="inlineStr">
-        <is>
-          <t>unique</t>
-        </is>
-      </c>
+          <t>Id</t>
+        </is>
+      </c>
+      <c r="C17" s="3" t="inlineStr"/>
       <c r="D17" s="3" t="inlineStr">
         <is>
-          <t>Role names are unique</t>
+          <t>Guid key</t>
         </is>
       </c>
       <c r="E17" s="3" t="inlineStr"/>
@@ -769,22 +774,22 @@
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
         <is>
-          <t>PK_UserRoles</t>
+          <t>UX_Roles_NormalizedName</t>
         </is>
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>UserId, RoleId</t>
+          <t>NormalizedName</t>
         </is>
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t>composite</t>
+          <t>unique</t>
         </is>
       </c>
       <c r="D18" s="3" t="inlineStr">
         <is>
-          <t>A user holds a role at most once</t>
+          <t>Role names are unique</t>
         </is>
       </c>
       <c r="E18" s="3" t="inlineStr"/>
@@ -792,18 +797,22 @@
     <row r="19">
       <c r="A19" s="3" t="inlineStr">
         <is>
-          <t>PK_RefreshTokens</t>
+          <t>PK_UserRoles</t>
         </is>
       </c>
       <c r="B19" s="3" t="inlineStr">
         <is>
-          <t>Id</t>
-        </is>
-      </c>
-      <c r="C19" s="3" t="inlineStr"/>
+          <t>UserId, RoleId</t>
+        </is>
+      </c>
+      <c r="C19" s="3" t="inlineStr">
+        <is>
+          <t>composite</t>
+        </is>
+      </c>
       <c r="D19" s="3" t="inlineStr">
         <is>
-          <t>Identity</t>
+          <t>A user holds a role at most once</t>
         </is>
       </c>
       <c r="E19" s="3" t="inlineStr"/>
@@ -811,85 +820,150 @@
     <row r="20">
       <c r="A20" s="3" t="inlineStr">
         <is>
-          <t>UX_RefreshTokens_TokenHash</t>
+          <t>IX_UserRoles_RoleId</t>
         </is>
       </c>
       <c r="B20" s="3" t="inlineStr">
         <is>
-          <t>TokenHash</t>
-        </is>
-      </c>
-      <c r="C20" s="3" t="inlineStr">
-        <is>
-          <t>unique</t>
-        </is>
-      </c>
+          <t>RoleId</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="n"/>
       <c r="D20" s="3" t="inlineStr">
         <is>
-          <t>A refresh looks up one token by its hash</t>
-        </is>
-      </c>
-      <c r="E20" s="3" t="inlineStr">
-        <is>
-          <t>RULE-23</t>
-        </is>
-      </c>
+          <t>"Who is an Administrator?", asked when the initial administrator is seeded. The composite key cannot seek on its second column alone</t>
+        </is>
+      </c>
+      <c r="E20" s="3" t="n"/>
     </row>
     <row r="21">
-      <c r="A21" s="2" t="inlineStr">
-        <is>
-          <t>Audit</t>
-        </is>
-      </c>
-      <c r="B21" s="3" t="inlineStr"/>
+      <c r="A21" s="3" t="inlineStr">
+        <is>
+          <t>PK_RefreshTokens</t>
+        </is>
+      </c>
+      <c r="B21" s="3" t="inlineStr">
+        <is>
+          <t>Id</t>
+        </is>
+      </c>
       <c r="C21" s="3" t="inlineStr"/>
-      <c r="D21" s="3" t="inlineStr"/>
+      <c r="D21" s="3" t="inlineStr">
+        <is>
+          <t>Identity</t>
+        </is>
+      </c>
       <c r="E21" s="3" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="3" t="inlineStr">
         <is>
-          <t>PK_AuditLog</t>
+          <t>UX_RefreshTokens_TokenHash</t>
         </is>
       </c>
       <c r="B22" s="3" t="inlineStr">
         <is>
-          <t>Id</t>
-        </is>
-      </c>
-      <c r="C22" s="3" t="inlineStr"/>
+          <t>TokenHash</t>
+        </is>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>unique</t>
+        </is>
+      </c>
       <c r="D22" s="3" t="inlineStr">
         <is>
-          <t>Identity</t>
-        </is>
-      </c>
-      <c r="E22" s="3" t="inlineStr"/>
+          <t>A refresh looks up one token by its hash</t>
+        </is>
+      </c>
+      <c r="E22" s="3" t="inlineStr">
+        <is>
+          <t>RULE-23</t>
+        </is>
+      </c>
     </row>
     <row r="23">
-      <c r="A23" s="2" t="inlineStr">
-        <is>
-          <t>Other indexes</t>
-        </is>
-      </c>
-      <c r="B23" s="3" t="inlineStr"/>
-      <c r="C23" s="3" t="inlineStr"/>
-      <c r="D23" s="3" t="inlineStr"/>
-      <c r="E23" s="3" t="inlineStr"/>
+      <c r="A23" s="3" t="inlineStr">
+        <is>
+          <t>IX_RefreshTokens_UserId</t>
+        </is>
+      </c>
+      <c r="B23" s="3" t="inlineStr">
+        <is>
+          <t>UserId</t>
+        </is>
+      </c>
+      <c r="C23" s="3" t="inlineStr">
+        <is>
+          <t>INCLUDE RevokedUtc, ExpiresUtc</t>
+        </is>
+      </c>
+      <c r="D23" s="3" t="inlineStr">
+        <is>
+          <t>Revoking every refresh token the user holds when a spent token is reused (AUTH-02), covered</t>
+        </is>
+      </c>
+      <c r="E23" s="3" t="inlineStr">
+        <is>
+          <t>RULE-23</t>
+        </is>
+      </c>
     </row>
     <row r="24">
-      <c r="A24" s="3" t="inlineStr">
-        <is>
-          <t>TBD</t>
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>Audit</t>
         </is>
       </c>
       <c r="B24" s="3" t="inlineStr"/>
       <c r="C24" s="3" t="inlineStr"/>
-      <c r="D24" s="3" t="inlineStr">
+      <c r="D24" s="3" t="inlineStr"/>
+      <c r="E24" s="3" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="3" t="inlineStr">
+        <is>
+          <t>PK_AuditLog</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="inlineStr">
+        <is>
+          <t>Id</t>
+        </is>
+      </c>
+      <c r="C25" s="3" t="inlineStr"/>
+      <c r="D25" s="3" t="inlineStr">
+        <is>
+          <t>Identity</t>
+        </is>
+      </c>
+      <c r="E25" s="3" t="inlineStr"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>Other indexes</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="inlineStr"/>
+      <c r="C26" s="3" t="inlineStr"/>
+      <c r="D26" s="3" t="inlineStr"/>
+      <c r="E26" s="3" t="inlineStr"/>
+    </row>
+    <row r="27">
+      <c r="A27" s="3" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="B27" s="3" t="inlineStr"/>
+      <c r="C27" s="3" t="inlineStr"/>
+      <c r="D27" s="3" t="inlineStr">
         <is>
           <t>Search, filtering and dashboard indexes are not designed yet</t>
         </is>
       </c>
-      <c r="E24" s="3" t="inlineStr"/>
+      <c r="E27" s="3" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -902,7 +976,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C11"/>
+  <dimension ref="A1:C13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="40" customWidth="1" min="1" max="1"/>
@@ -1002,31 +1076,33 @@
       <c r="C7" s="3" t="inlineStr"/>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>Concurrency</t>
-        </is>
-      </c>
-      <c r="B8" s="3" t="inlineStr"/>
-      <c r="C8" s="3" t="inlineStr"/>
+      <c r="A8" s="3" t="inlineStr">
+        <is>
+          <t>Users.AccessFailedCount</t>
+        </is>
+      </c>
+      <c r="B8" s="3" t="inlineStr">
+        <is>
+          <t>Defaults to 0. Counts consecutive failed sign-ins toward the 5-attempt lockout (AUTH-01)</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="3" t="inlineStr">
         <is>
-          <t>Assets.RowVersion</t>
+          <t>Users.CreatedUtc, RefreshTokens.CreatedUtc</t>
         </is>
       </c>
       <c r="B9" s="3" t="inlineStr">
         <is>
-          <t>Concurrency token for edits</t>
-        </is>
-      </c>
-      <c r="C9" s="3" t="inlineStr"/>
+          <t>Default to SYSUTCDATETIME()</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Check constraints</t>
+          <t>Concurrency</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr"/>
@@ -1035,15 +1111,37 @@
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
         <is>
-          <t>TBD</t>
+          <t>Assets.RowVersion</t>
         </is>
       </c>
       <c r="B11" s="3" t="inlineStr">
         <is>
+          <t>Concurrency token for edits</t>
+        </is>
+      </c>
+      <c r="C11" s="3" t="inlineStr"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>Check constraints</t>
+        </is>
+      </c>
+      <c r="B12" s="3" t="inlineStr"/>
+      <c r="C12" s="3" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="3" t="inlineStr">
+        <is>
+          <t>TBD</t>
+        </is>
+      </c>
+      <c r="B13" s="3" t="inlineStr">
+        <is>
           <t>Not designed yet</t>
         </is>
       </c>
-      <c r="C11" s="3" t="inlineStr"/>
+      <c r="C13" s="3" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -1213,10 +1311,14 @@
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>TBD</t>
-        </is>
-      </c>
-      <c r="C10" s="3" t="inlineStr"/>
+          <t>CASCADE</t>
+        </is>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>Sessions are worthless without their user, and leaving them would leave live tokens pointing nowhere</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="3" t="inlineStr">
@@ -1241,6 +1343,79 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="100" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Script</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Contents</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>0001_CreateSchema.sql</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>The identity tables: Users, Roles, UserRoles and RefreshTokens, with their keys, indexes and defaults. The rest of the model arrives in later scripts as it is built.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>0002_SeedRoles.sql</t>
+        </is>
+      </c>
+      <c r="B3" s="3" t="inlineStr">
+        <is>
+          <t>The four roles, with fixed literal ids rather than NEWID(), so every environment has the same ids and a UserRoles row from one database means the same thing in another. Written as a MERGE, so re-running is safe.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="3" t="inlineStr">
+        <is>
+          <t>API startup</t>
+        </is>
+      </c>
+      <c r="B4" s="3" t="inlineStr">
+        <is>
+          <t>The initial administrator account. Not a script, because only Identity services can produce a valid password hash. When no user has the configured email, it creates one with the Administrator role; otherwise it does nothing. The email and password are supplied as secrets, never committed in appsettings.json.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>Migration is a separate step (AssetHub.Migrator), never a side effect of the API starting. DbUp journals every applied script in dbo.SchemaVersions and runs each exactly once, in name order, each in its own transaction. Scripts are append-only: a mistake is fixed by a new script, never by editing one that has already run.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>